<commit_message>
feat: upgrade slide generator agent with dynamic tech stack, sentence case rules, borderless images & multi-lesson support
</commit_message>
<xml_diff>
--- a/output/pms/Quản_lý_phiên_bản_với_GIT/PM_Generated_IT105.xlsx
+++ b/output/pms/Quản_lý_phiên_bản_với_GIT/PM_Generated_IT105.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="PM_Syllabus" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PM_Syllabus" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -230,8 +230,8 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -687,7 +687,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Xây dựng sản phẩm dự án cuối khóa sử dụng Git 2.45+, GitHub Web &amp; CLI, Git Flow Standard Branching Model, SSH / GPG Standard Authentication (Conventional Commits, Clean Git History, .gitignore Best Practices)</t>
+          <t>Xây dựng sản phẩm dự án cuối khóa sử dụng Git CLI 2.45+, GitHub Cloud (Conventional Commits, Git Flow, Semantic Branching)</t>
         </is>
       </c>
       <c r="C3" s="8" t="n"/>
@@ -769,37 +769,37 @@
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>Session 01 - Định hướng môn học Git</t>
+          <t>Session 01 - Định hướng khóa học &amp; Lộ trình Git Version Control</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Lesson 01: Giới thiệu môn học và CLO</t>
+          <t>Lesson 01: Tổng quan nội dung &amp; Lộ trình môn học</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Ý nghĩa Git; Chuẩn đầu ra CLO; Cách đánh giá</t>
+          <t>Giới thiệu mục tiêu môn học IT-105; Lộ trình 10 buổi học quản lý dự án Web responsive và framework JavaScript; Chuẩn đầu ra CLO, PLO; Quy định đánh giá và thi thực hành cuối môn.</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Hiểu rõ cấu trúc môn học và tiêu chí đánh giá.</t>
+          <t>Trình bày được toàn bộ cấu trúc môn học, các mốc đánh giá và mục tiêu đầu ra cần đạt được.</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>CẤM: commit, push, clone, branch, merge, SSH</t>
+          <t>CẤM: Gõ lệnh Git CLI, cài đặt Git, thao tác terminal, git init, git add.</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>ĐÃ HỌC: Chưa có.</t>
+          <t>ĐÃ HỌC: Không (Bài mở đầu).</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>Git 2.45+, GitHub Web &amp; CLI, Git Flow Standard Branching Model, SSH / GPG Standard Authentication (Conventional Commits, Clean Git History, .gitignore Best Practices)</t>
+          <t>Git CLI 2.45+, GitHub Cloud (Conventional Commits, Git Flow, Semantic Branching)</t>
         </is>
       </c>
     </row>
@@ -810,120 +810,120 @@
       <c r="D7" s="12" t="n"/>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Lesson 02: Phương pháp tự học Git bằng AI</t>
+          <t>Lesson 02: Phương pháp học tập hiệu quả</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Tự học Git; Ứng dụng LLM; Cách tra cứu nhanh</t>
+          <t>Phương pháp tự học chủ động; Ứng dụng Prompt Engineering với LLMs (ChatGPT/Claude) để sinh tự động câu lệnh tra cứu Git, giải thích lỗi terminal và tóm tắt tài liệu; Kỹ năng quản lý thời gian làm việc nhóm.</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Biết cách tối ưu hóa tốc độ tự học qua LLM.</t>
+          <t>Áp dụng được kỹ thuật đặt câu hỏi (Prompting) với AI để sinh cú pháp lệnh Git và giải quyết lỗi cơ bản trong quá trình học.</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>CẤM: commit, push, clone, branch, merge, SSH</t>
+          <t>CẤM: Tạo repository, git commit, git push, git merge.</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>ĐÃ HỌC: Lộ trình môn học.</t>
+          <t>ĐÃ HỌC: Định hướng lộ trình môn học.</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>Git 2.45+, GitHub Web &amp; CLI, Git Flow Standard Branching Model, SSH / GPG Standard Authentication (Conventional Commits, Clean Git History, .gitignore Best Practices)</t>
+          <t>Git CLI 2.45+, GitHub Cloud (Conventional Commits, Git Flow, Semantic Branching)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="13" t="n"/>
+      <c r="B8" s="13" t="n"/>
+      <c r="C8" s="13" t="n"/>
+      <c r="D8" s="13" t="n"/>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Lesson 03: Demo sản phẩm thực tế &amp; Kỳ vọng đầu ra</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Demo quy trình quản lý dự án Web responsive thực tế xây dựng trên framework JavaScript; Demo luồng làm việc nhóm (Git Flow, Pull Request, Code Review); Tiêu chuẩn kho lưu trữ mã nguồn chuẩn doanh nghiệp.</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Phân tích được sản phẩm thực tế cần đạt được sau khóa học và các tiêu chí của kho chứa mã nguồn dự án framework đạt chuẩn doanh nghiệp.</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>CẤM: Thực hành gõ lệnh Git, cài đặt Git Bash.</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>ĐÃ HỌC: Lộ trình môn học, Phương pháp học tập với AI.</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>Git CLI 2.45+, GitHub Cloud (Conventional Commits, Git Flow, Semantic Branching)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Session 02</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Lý thuyết</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>THEORY</t>
         </is>
       </c>
-      <c r="D8" s="11" t="inlineStr">
-        <is>
-          <t>Session 02 - Kiến trúc và thiết lập Git cục bộ</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>Lesson 01: Mô hình quản lý phiên bản Git</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>Vấn đề lưu trữ; Giải pháp Git; Kiến trúc 3 vùng</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>Phân biệt được ba vùng dữ liệu của Git.</t>
-        </is>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>CẤM: git config, git init, commit</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>ĐÃ HỌC: Lộ trình môn học Git.</t>
-        </is>
-      </c>
-      <c r="J8" s="5" t="inlineStr">
-        <is>
-          <t>Git 2.45+, GitHub Web &amp; CLI, Git Flow Standard Branching Model, SSH / GPG Standard Authentication (Conventional Commits, Clean Git History, .gitignore Best Practices)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="13" t="n"/>
-      <c r="B9" s="13" t="n"/>
-      <c r="C9" s="13" t="n"/>
-      <c r="D9" s="13" t="n"/>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Session 02 - Cấu trúc kho chứa &amp; Lệnh Git CLI cơ bản</t>
+        </is>
+      </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Lesson 02: Cài đặt và thiết lập Git ban đầu</t>
+          <t>Lesson 01: Tổng quan về hệ thống quản lý phiên bản Git</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Cài đặt Git; git config; user email; user name</t>
+          <t>Khái niệm Version Control System (VCS); Phân biệt Centralized VCS và Distributed VCS (DVCS); Nguyên lý lưu trữ và sinh dữ liệu dạng Snapshot của Git; Lợi ích của Git CLI 2.45+ trong quản lý dự án phần mềm.</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Thiết lập thành công thông tin danh tính Git.</t>
+          <t>Phân biệt được VCS tập trung và phân tán; Mô tả được cơ chế Snapshot và ưu điểm của Git CLI.</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>CẤM: git init, commit, remote</t>
+          <t>CẤM: GitHub Remote, git push, git branch, git merge.</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>ĐÃ HỌC: Kiến trúc 3 vùng Git.</t>
+          <t>ĐÃ HỌC: Định hướng khóa học.</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>Git 2.45+, GitHub Web &amp; CLI, Git Flow Standard Branching Model, SSH / GPG Standard Authentication (Conventional Commits, Clean Git History, .gitignore Best Practices)</t>
+          <t>Git CLI 2.45+, GitHub Cloud (Conventional Commits, Git Flow, Semantic Branching)</t>
         </is>
       </c>
     </row>
@@ -934,136 +934,104 @@
       <c r="D10" s="12" t="n"/>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Lesson 03: Khởi tạo kho lưu trữ cục bộ</t>
+          <t>Lesson 02: Cài đặt &amp; Cấu hình môi trường Git CLI</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Thư mục dự án; git init; Thư mục .git</t>
+          <t>Cài đặt Git CLI 2.45+ trên hệ điều hành; Cấu hình thông tin người dùng toàn cục git config --global user.name và user.email; Cấu hình trình biên tập mặc định; Tích hợp Git terminal vào VS Code.</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Khởi tạo thành công repository cục bộ.</t>
+          <t>Cài đặt thành công Git CLI 2.45+; Cấu hình chính xác danh tính lập trình viên trên Git CLI và tích hợp vào VS Code.</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>CẤM: git add, commit, push</t>
+          <t>CẤM: GitHub Remote, SSH key, git push, git branch.</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>ĐÃ HỌC: Thiết lập git config.</t>
+          <t>ĐÃ HỌC: Nguyên lý hoạt động của Git.</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>Git 2.45+, GitHub Web &amp; CLI, Git Flow Standard Branching Model, SSH / GPG Standard Authentication (Conventional Commits, Clean Git History, .gitignore Best Practices)</t>
+          <t>Git CLI 2.45+, GitHub Cloud (Conventional Commits, Git Flow, Semantic Branching)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="14" t="inlineStr">
-        <is>
-          <t>Session 03</t>
-        </is>
-      </c>
-      <c r="B11" s="14" t="inlineStr">
-        <is>
-          <t>Thực hành</t>
-        </is>
-      </c>
-      <c r="C11" s="14" t="inlineStr">
-        <is>
-          <t>PRACTICE</t>
-        </is>
-      </c>
-      <c r="D11" s="15" t="inlineStr">
-        <is>
-          <t>Session 03 - Thực hành khởi tạo dự án Git</t>
-        </is>
-      </c>
-      <c r="E11" s="16" t="inlineStr">
-        <is>
-          <t>Session 03 - Thực hành khởi tạo dự án Git</t>
-        </is>
-      </c>
-      <c r="F11" s="16" t="inlineStr">
-        <is>
-          <t>git init; git config; git status</t>
-        </is>
-      </c>
-      <c r="G11" s="16" t="inlineStr">
-        <is>
-          <t>Thực hiện thành thạo khởi tạo local repository.</t>
-        </is>
-      </c>
-      <c r="H11" s="16" t="inlineStr">
-        <is>
-          <t>CẤM: git add, commit, remote, push, branch</t>
-        </is>
-      </c>
-      <c r="I11" s="16" t="inlineStr">
-        <is>
-          <t>ĐÃ HỌC: Cấu hình Git, git init.</t>
-        </is>
-      </c>
-      <c r="J11" s="16" t="inlineStr">
-        <is>
-          <t>Git 2.45+, GitHub Web &amp; CLI, Git Flow Standard Branching Model, SSH / GPG Standard Authentication (Conventional Commits, Clean Git History, .gitignore Best Practices)</t>
+      <c r="A11" s="12" t="n"/>
+      <c r="B11" s="12" t="n"/>
+      <c r="C11" s="12" t="n"/>
+      <c r="D11" s="12" t="n"/>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Lesson 03: Khởi tạo kho chứa &amp; Kiến trúc 3 vùng dữ liệu</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Lệnh git init để sinh thư mục ẩn .git; Kiến trúc 3 vùng làm việc: Working Directory (Thư mục làm việc), Staging Area (Vùng chờ), Local Repository (Kho chứa cục bộ); Lệnh kiểm tra trạng thái git status.</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Khởi tạo được kho chứa cục bộ bằng git init; Phân tích được luồng chuyển đổi dữ liệu giữa 3 vùng làm việc và kiểm tra trạng thái bằng git status.</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>CẤM: git push, git pull, git branch, GitHub Cloud.</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>ĐÃ HỌC: Cài đặt &amp; cấu hình Git CLI.</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>Git CLI 2.45+, GitHub Cloud (Conventional Commits, Git Flow, Semantic Branching)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>Session 04</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>Lý thuyết</t>
-        </is>
-      </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>THEORY</t>
-        </is>
-      </c>
-      <c r="D12" s="11" t="inlineStr">
-        <is>
-          <t>Session 04 - Làm việc với commits và history</t>
-        </is>
-      </c>
+      <c r="A12" s="12" t="n"/>
+      <c r="B12" s="12" t="n"/>
+      <c r="C12" s="12" t="n"/>
+      <c r="D12" s="12" t="n"/>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Lesson 01: Đưa tệp tin vào staging area</t>
+          <t>Lesson 04: Quản lý vùng chờ Staging &amp; Tập tin loại trừ .gitignore cho dự án Web framework</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>git add; Trạng thái tệp; Staged; Tracked</t>
+          <t>Lệnh git add (git add &lt;file&gt;, git add .); Đưa file vào Staging Area; Cú pháp và quy tắc viết file .gitignore cho các project Web responsive dùng JavaScript framework; Bỏ qua thư mục node_modules, build artifacts và tập tin môi trường nhạy cảm (.env).</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Đưa tệp tin vào trạng thái staged thành công.</t>
+          <t>Đưa được tập tin vào Staging Area; Tạo và cấu hình chính xác file .gitignore để loại trừ các tệp tin không mong muốn của project framework khỏi Git.</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>CẤM: git commit, git log, remote</t>
+          <t>CẤM: git push, git remote, git branch, Pull Request.</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>ĐÃ HỌC: git init, git config, git status.</t>
+          <t>ĐÃ HỌC: git init, 3 vùng dữ liệu, git status.</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>Git 2.45+, GitHub Web &amp; CLI, Git Flow Standard Branching Model, SSH / GPG Standard Authentication (Conventional Commits, Clean Git History, .gitignore Best Practices)</t>
+          <t>Git CLI 2.45+, GitHub Cloud (Conventional Commits, Git Flow, Semantic Branching)</t>
         </is>
       </c>
     </row>
@@ -1074,172 +1042,172 @@
       <c r="D13" s="13" t="n"/>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Lesson 02: Tạo commit và quy chuẩn thông điệp</t>
+          <t>Lesson 05: Ghi nhận phiên bản Commit &amp; Chuẩn Conventional Commits</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>git commit -m; Conventional Commits</t>
+          <t>Lệnh git commit -m; Quy chuẩn đặt thông điệp commit Conventional Commits (feat, fix, docs, style, refactor); Sử dụng AI để sinh câu thông điệp commit chuẩn xác; Lệnh xem lịch sử commit git log, git log --oneline.</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Viết thông điệp commit đúng chuẩn Conventional.</t>
+          <t>Thực hiện lưu phiên bản mã nguồn với git commit theo đúng chuẩn Conventional Commits; Truy vấn lịch sử thay đổi mã nguồn bằng git log.</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>CẤM: git log, .gitignore, remote</t>
+          <t>CẤM: git push, git remote, git branch, git merge, GitHub.</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>ĐÃ HỌC: git add.</t>
+          <t>ĐÃ HỌC: git init, git status, git add, .gitignore.</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>Git 2.45+, GitHub Web &amp; CLI, Git Flow Standard Branching Model, SSH / GPG Standard Authentication (Conventional Commits, Clean Git History, .gitignore Best Practices)</t>
+          <t>Git CLI 2.45+, GitHub Cloud (Conventional Commits, Git Flow, Semantic Branching)</t>
         </is>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="12" t="n"/>
-      <c r="B14" s="12" t="n"/>
-      <c r="C14" s="12" t="n"/>
-      <c r="D14" s="12" t="n"/>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>Lesson 03: Quản lý lịch sử và bỏ qua tệp</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>git log; Tùy chọn log; Tệp .gitignore</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>Xem lịch sử thay đổi và cấu hình .gitignore.</t>
-        </is>
-      </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>CẤM: remote, push, GPG, branch</t>
-        </is>
-      </c>
-      <c r="I14" s="5" t="inlineStr">
-        <is>
-          <t>ĐÃ HỌC: git commit.</t>
-        </is>
-      </c>
-      <c r="J14" s="5" t="inlineStr">
-        <is>
-          <t>Git 2.45+, GitHub Web &amp; CLI, Git Flow Standard Branching Model, SSH / GPG Standard Authentication (Conventional Commits, Clean Git History, .gitignore Best Practices)</t>
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>Session 03</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>Thực hành</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>PRACTICE</t>
+        </is>
+      </c>
+      <c r="D14" s="15" t="inlineStr">
+        <is>
+          <t>Session 03 - Thực hành Quản lý phiên bản mã nguồn cục bộ dự án JavaScript</t>
+        </is>
+      </c>
+      <c r="E14" s="16" t="inlineStr">
+        <is>
+          <t>Session 03 - Thực hành Quản lý phiên bản mã nguồn cục bộ dự án JavaScript</t>
+        </is>
+      </c>
+      <c r="F14" s="16" t="inlineStr">
+        <is>
+          <t>Luyện tập quản lý mã nguồn Web responsive xây dựng với framework JavaScript; Khởi tạo Git repository cục bộ với git init; Cấu hình file .gitignore loại bỏ các tệp rác dự án framework; Đưa mã nguồn vào Staging Area bằng git add; Thực hiện chuỗi commit chuẩn Conventional Commits cho từng tính năng giao diện responsive; Tra cứu lịch sử phiên bản với git log; Luyện tập ứng dụng AI (Prompt Engineering) để sinh thông điệp commit message chuẩn doanh nghiệp.</t>
+        </is>
+      </c>
+      <c r="G14" s="16" t="inlineStr">
+        <is>
+          <t>Luyện tập và khởi tạo thành công lịch sử phiên bản cục bộ cho dự án Web responsive sử dụng JavaScript framework; Viết đúng thông điệp commit theo chuẩn Conventional Commits và sinh file .gitignore hoàn chỉnh.</t>
+        </is>
+      </c>
+      <c r="H14" s="16" t="inlineStr">
+        <is>
+          <t>CẤM: GitHub Cloud, git remote, git push, git pull, git branch, git merge.</t>
+        </is>
+      </c>
+      <c r="I14" s="16" t="inlineStr">
+        <is>
+          <t>ĐÃ HỌC: Lệnh Git CLI cơ bản (git init, git status, git add, git commit, .gitignore cho dự án framework, git log), Kỹ thuật Prompt Engineering sinh commit message.</t>
+        </is>
+      </c>
+      <c r="J14" s="16" t="inlineStr">
+        <is>
+          <t>Git CLI 2.45+, GitHub Cloud (Conventional Commits, Git Flow, Semantic Branching)</t>
         </is>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="14" t="inlineStr">
-        <is>
-          <t>Session 05</t>
-        </is>
-      </c>
-      <c r="B15" s="14" t="inlineStr">
-        <is>
-          <t>Thực hành</t>
-        </is>
-      </c>
-      <c r="C15" s="14" t="inlineStr">
-        <is>
-          <t>PRACTICE</t>
-        </is>
-      </c>
-      <c r="D15" s="15" t="inlineStr">
-        <is>
-          <t>Session 05 - Thực hành commit và quản lý tệp</t>
-        </is>
-      </c>
-      <c r="E15" s="16" t="inlineStr">
-        <is>
-          <t>Session 05 - Thực hành commit và quản lý tệp</t>
-        </is>
-      </c>
-      <c r="F15" s="16" t="inlineStr">
-        <is>
-          <t>git add; git commit; .gitignore; git log</t>
-        </is>
-      </c>
-      <c r="G15" s="16" t="inlineStr">
-        <is>
-          <t>Lưu trữ phiên bản mã nguồn đúng quy chuẩn.</t>
-        </is>
-      </c>
-      <c r="H15" s="16" t="inlineStr">
-        <is>
-          <t>CẤM: remote, push, SSH, GPG, branch, merge</t>
-        </is>
-      </c>
-      <c r="I15" s="16" t="inlineStr">
-        <is>
-          <t>ĐÃ HỌC: git add, git commit, git log, .gitignore.</t>
-        </is>
-      </c>
-      <c r="J15" s="16" t="inlineStr">
-        <is>
-          <t>Git 2.45+, GitHub Web &amp; CLI, Git Flow Standard Branching Model, SSH / GPG Standard Authentication (Conventional Commits, Clean Git History, .gitignore Best Practices)</t>
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Session 04</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>Lý thuyết</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>THEORY</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Session 04 - Đồng bộ mã nguồn với GitHub Cloud &amp; Remote Repositories</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Lesson 01: Tổng quan GitHub Cloud &amp; Cấu hình phương thức xác thực SSH/PAT</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Khái niệm Remote Repository và GitHub Cloud; Khởi tạo tài khoản GitHub; Sinh khóa SSH Key (ssh-keygen) và liên kết Public Key với GitHub; Cấu hình Personal Access Token (PAT) cho Git CLI.</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Sinh và cấu hình thành công SSH Key / PAT để kết nối xác thực an toàn giữa Git CLI và GitHub Cloud.</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>CẤM: git branch, git merge, Pull Request.</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>ĐÃ HỌC: Git CLI cục bộ, git commit, git log.</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>Git CLI 2.45+, GitHub Cloud (Conventional Commits, Git Flow, Semantic Branching)</t>
         </is>
       </c>
     </row>
     <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
-        <is>
-          <t>Session 06</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>Lý thuyết</t>
-        </is>
-      </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>THEORY</t>
-        </is>
-      </c>
-      <c r="D16" s="11" t="inlineStr">
-        <is>
-          <t>Session 06 - Kết nối Remote và bảo mật GitHub</t>
-        </is>
-      </c>
+      <c r="A16" s="12" t="n"/>
+      <c r="B16" s="12" t="n"/>
+      <c r="C16" s="12" t="n"/>
+      <c r="D16" s="12" t="n"/>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Lesson 01: Tạo kho lưu trữ trên GitHub</t>
+          <t>Lesson 02: Liên kết kho chứa từ xa Remote &amp; Đẩy mã nguồn git push</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>GitHub; Remote repository; GitHub Web</t>
+          <t>Khởi tạo kho chứa mới (Remote Repository) trên GitHub Cloud; Lệnh git remote add origin &lt;url&gt;; Kiểm tra danh sách remote git remote -v; Đẩy commit từ local lên remote bằng git push -u origin main.</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Khởi tạo thành công repository trên GitHub Web.</t>
+          <t>Khởi tạo thành công Remote Repository trên GitHub; Liên kết kho chứa local với remote và đẩy mã nguồn lên GitHub Cloud.</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>CẤM: SSH key, commit signature, push</t>
+          <t>CẤM: git branch, git merge, PR review.</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>ĐÃ HỌC: Lưu trữ Git cục bộ.</t>
+          <t>ĐÃ HỌC: Cấu hình SSH/PAT GitHub, git commit.</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>Git 2.45+, GitHub Web &amp; CLI, Git Flow Standard Branching Model, SSH / GPG Standard Authentication (Conventional Commits, Clean Git History, .gitignore Best Practices)</t>
+          <t>Git CLI 2.45+, GitHub Cloud (Conventional Commits, Git Flow, Semantic Branching)</t>
         </is>
       </c>
     </row>
@@ -1250,172 +1218,156 @@
       <c r="D17" s="13" t="n"/>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Lesson 02: Thiết lập bảo mật SSH và GPG</t>
+          <t>Lesson 03: Sao chép kho chứa git clone &amp; Tải mã nguồn git fetch, git pull</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>SSH keygen; GitHub SSH; GPG signature</t>
+          <t>Lệnh git clone &lt;url&gt; để tải dự án từ GitHub về máy mới; Khái niệm Tracking Branch; Lệnh git fetch để kiểm tra cập nhật remote; Lệnh git pull để tải và hợp nhất thay đổi; Phân biệt sự khác nhau giữa git fetch và git pull.</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Xác thực thành công SSH và GPG trên GitHub.</t>
+          <t>Thực hiện sao chép kho chứa với git clone; Phân biệt rõ sự khác nhau giữa git fetch và git pull; Cấu hình thành công đồng bộ mã nguồn mới nhất từ GitHub.</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>CẤM: git remote add, git push</t>
+          <t>CẤM: Phân nhánh nâng cao, Git Flow, Pull Request.</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>ĐÃ HỌC: Đăng ký tài khoản GitHub.</t>
+          <t>ĐÃ HỌC: git remote, git push, SSH GitHub.</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>Git 2.45+, GitHub Web &amp; CLI, Git Flow Standard Branching Model, SSH / GPG Standard Authentication (Conventional Commits, Clean Git History, .gitignore Best Practices)</t>
+          <t>Git CLI 2.45+, GitHub Cloud (Conventional Commits, Git Flow, Semantic Branching)</t>
         </is>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="12" t="n"/>
-      <c r="B18" s="12" t="n"/>
-      <c r="C18" s="12" t="n"/>
-      <c r="D18" s="12" t="n"/>
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Session 05</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Lý thuyết</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>THEORY</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>Session 05 - Quản lý phân nhánh Git Branch &amp; Kỹ thuật Xử lý xung đột mã nguồn</t>
+        </is>
+      </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Lesson 03: Liên kết và đồng bộ lên GitHub</t>
+          <t>Lesson 01: Khái niệm phân nhánh &amp; Chiến lược Semantic Branching</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>git remote add; git push; git clone; git pull</t>
+          <t>Bản chất của Branch trong Git (con trỏ chỉ đến commit); Con trỏ HEAD; Lệnh git branch, git switch -c, git checkout -b; Quy chuẩn đặt tên nhánh Semantic Branching (feature/responsive-layout, fix/header-bug).</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Đẩy mã nguồn cục bộ lên GitHub thành công.</t>
+          <t>Giải thích được cơ chế hoạt động của nhánh và con trỏ HEAD; Tạo và chuyển đổi nhánh thành thạo theo quy chuẩn Semantic Branching.</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>CẤM: branch, merge, PR</t>
+          <t>CẤM: git merge, Merge Conflict, Pull Request.</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>ĐÃ HỌC: Xác thực SSH/GPG.</t>
+          <t>ĐÃ HỌC: Git CLI, GitHub Remote.</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>Git 2.45+, GitHub Web &amp; CLI, Git Flow Standard Branching Model, SSH / GPG Standard Authentication (Conventional Commits, Clean Git History, .gitignore Best Practices)</t>
+          <t>Git CLI 2.45+, GitHub Cloud (Conventional Commits, Git Flow, Semantic Branching)</t>
         </is>
       </c>
     </row>
     <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="14" t="inlineStr">
-        <is>
-          <t>Session 07</t>
-        </is>
-      </c>
-      <c r="B19" s="14" t="inlineStr">
-        <is>
-          <t>Thực hành</t>
-        </is>
-      </c>
-      <c r="C19" s="14" t="inlineStr">
-        <is>
-          <t>PRACTICE</t>
-        </is>
-      </c>
-      <c r="D19" s="15" t="inlineStr">
-        <is>
-          <t>Session 07 - Thực hành đồng bộ mã nguồn GitHub</t>
-        </is>
-      </c>
-      <c r="E19" s="16" t="inlineStr">
-        <is>
-          <t>Session 07 - Thực hành đồng bộ mã nguồn GitHub</t>
-        </is>
-      </c>
-      <c r="F19" s="16" t="inlineStr">
-        <is>
-          <t>SSH key; git remote; git push; git pull</t>
-        </is>
-      </c>
-      <c r="G19" s="16" t="inlineStr">
-        <is>
-          <t>Đẩy và kéo mã nguồn từ GitHub thành thạo.</t>
-        </is>
-      </c>
-      <c r="H19" s="16" t="inlineStr">
-        <is>
-          <t>CẤM: branch, merge conflict, Git Flow</t>
-        </is>
-      </c>
-      <c r="I19" s="16" t="inlineStr">
-        <is>
-          <t>ĐÃ HỌC: SSH key, GitHub, remote, push, pull.</t>
-        </is>
-      </c>
-      <c r="J19" s="16" t="inlineStr">
-        <is>
-          <t>Git 2.45+, GitHub Web &amp; CLI, Git Flow Standard Branching Model, SSH / GPG Standard Authentication (Conventional Commits, Clean Git History, .gitignore Best Practices)</t>
+      <c r="A19" s="12" t="n"/>
+      <c r="B19" s="12" t="n"/>
+      <c r="C19" s="12" t="n"/>
+      <c r="D19" s="12" t="n"/>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Lesson 02: Hợp nhất nhánh Fast-Forward &amp; 3-Way Merge</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Lệnh git merge &lt;branch-name&gt;; Hợp nhất kiểu Fast-Forward Merge (không có commit mới trên nhánh chính); Hợp nhất kiểu 3-Way Merge (tạo merge commit); Lệnh xóa nhánh git branch -d.</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>Thực hiện hợp nhất nhánh thành công; Phân biệt được Fast-Forward Merge và 3-Way Merge.</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>CẤM: Merge Conflict, Pull Request trên GitHub.</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>ĐÃ HỌC: Tạo và chuyển đổi nhánh git branch.</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>Git CLI 2.45+, GitHub Cloud (Conventional Commits, Git Flow, Semantic Branching)</t>
         </is>
       </c>
     </row>
     <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="10" t="inlineStr">
-        <is>
-          <t>Session 08</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>Lý thuyết</t>
-        </is>
-      </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>THEORY</t>
-        </is>
-      </c>
-      <c r="D20" s="11" t="inlineStr">
-        <is>
-          <t>Session 08 - Phân nhánh và quy trình Git Flow</t>
-        </is>
-      </c>
+      <c r="A20" s="12" t="n"/>
+      <c r="B20" s="12" t="n"/>
+      <c r="C20" s="12" t="n"/>
+      <c r="D20" s="12" t="n"/>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Lesson 01: Quản lý nhánh cục bộ và từ xa</t>
+          <t>Lesson 03: Kỹ thuật Xử lý xung đột mã nguồn Merge Conflict &amp; Debugging</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>git branch; git checkout; git switch; branch remote</t>
+          <t>Nguyên nhân gây ra Merge Conflict (thay đổi cùng dòng code giao diện responsive trên các nhánh khác nhau); Dấu hiệu nhận biết conflict (&lt;&lt;&lt;&lt;&lt;&lt;&lt;, =======, &gt;&gt;&gt;&gt;&gt;&gt;&gt;); Kỹ thuật debugging xung đột trong VS Code (Accept Current, Accept Incoming, Accept Both); Đóng commit hợp nhất sau khi sửa conflict.</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Tạo, chuyển đổi và quản lý các nhánh cục bộ.</t>
+          <t>Phát hiện và nhận diện đúng vị trí xung đột mã nguồn; Thực hiện debugging và giải quyết xung đột thành công trên VS Code để hoàn tất commit hợp nhất.</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>CẤM: git merge, conflict, Git Flow</t>
+          <t>CẤM: Git Flow mô hình doanh nghiệp, PR Review.</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>ĐÃ HỌC: Remote push, pull.</t>
+          <t>ĐÃ HỌC: git branch, git merge.</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>Git 2.45+, GitHub Web &amp; CLI, Git Flow Standard Branching Model, SSH / GPG Standard Authentication (Conventional Commits, Clean Git History, .gitignore Best Practices)</t>
+          <t>Git CLI 2.45+, GitHub Cloud (Conventional Commits, Git Flow, Semantic Branching)</t>
         </is>
       </c>
     </row>
@@ -1426,200 +1378,468 @@
       <c r="D21" s="13" t="n"/>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Lesson 02: Tích hợp và xử lý xung đột</t>
+          <t>Lesson 04: Tạm lưu thay đổi với Git Stash</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>git merge; Merge Conflict; Sửa conflict</t>
+          <t>Lý do cần lưu tạm công việc chưa commit; Lệnh git stash push; Lệnh git stash list; Khôi phục thay đổi với git stash apply và git stash pop; Xóa stash với git stash drop và git stash clear.</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Giải quyết xung đột khi hợp nhất các nhánh.</t>
+          <t>Thực hiện lưu trữ và khôi phục trạng thái làm việc dở dang bằng các lệnh git stash mà không tạo commit rác.</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>CẤM: Git Flow branching model</t>
+          <t>CẤM: Pull Request, Code Review.</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>ĐÃ HỌC: Quản lý nhánh.</t>
+          <t>ĐÃ HỌC: Phân nhánh, hợp nhất nhánh, xử lý xung đột.</t>
         </is>
       </c>
       <c r="J21" s="5" t="inlineStr">
         <is>
-          <t>Git 2.45+, GitHub Web &amp; CLI, Git Flow Standard Branching Model, SSH / GPG Standard Authentication (Conventional Commits, Clean Git History, .gitignore Best Practices)</t>
+          <t>Git CLI 2.45+, GitHub Cloud (Conventional Commits, Git Flow, Semantic Branching)</t>
         </is>
       </c>
     </row>
     <row r="22" ht="24" customHeight="1">
-      <c r="A22" s="12" t="n"/>
-      <c r="B22" s="12" t="n"/>
-      <c r="C22" s="12" t="n"/>
-      <c r="D22" s="12" t="n"/>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>Lesson 03: Quy trình Git Flow và Pull Request</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>Git Flow; main; develop; feature; PR</t>
-        </is>
-      </c>
-      <c r="G22" s="5" t="inlineStr">
-        <is>
-          <t>Triển khai được quy trình phân nhánh chuẩn.</t>
-        </is>
-      </c>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>CẤM: Không có.</t>
-        </is>
-      </c>
-      <c r="I22" s="5" t="inlineStr">
-        <is>
-          <t>ĐÃ HỌC: Hợp nhất nhánh.</t>
-        </is>
-      </c>
-      <c r="J22" s="5" t="inlineStr">
-        <is>
-          <t>Git 2.45+, GitHub Web &amp; CLI, Git Flow Standard Branching Model, SSH / GPG Standard Authentication (Conventional Commits, Clean Git History, .gitignore Best Practices)</t>
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>Session 06</t>
+        </is>
+      </c>
+      <c r="B22" s="14" t="inlineStr">
+        <is>
+          <t>Thực hành</t>
+        </is>
+      </c>
+      <c r="C22" s="14" t="inlineStr">
+        <is>
+          <t>PRACTICE</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>Session 06 - Thực hành Phân nhánh, Đồng bộ GitHub &amp; Xử lý xung đột mã nguồn</t>
+        </is>
+      </c>
+      <c r="E22" s="16" t="inlineStr">
+        <is>
+          <t>Session 06 - Thực hành Phân nhánh, Đồng bộ GitHub &amp; Xử lý xung đột mã nguồn</t>
+        </is>
+      </c>
+      <c r="F22" s="16" t="inlineStr">
+        <is>
+          <t>Luyện tập chia nhánh tính năng cho dự án Web responsive xây dựng với framework JavaScript (ví dụ: feature/responsive-nav, feature/card-component); Thực hiện commit riêng biệt trên từng nhánh; Cố tình tạo tình huống xung đột mã nguồn (Merge Conflict) trên file cấu hình hoặc giao diện giữa 2 nhánh; Luyện tập debugging và giải quyết xung đột trong VS Code; Thực hành git stash khi cần chuyển nhánh gấp để xử lý hotfix; Đẩy các nhánh tính năng lên GitHub Cloud.</t>
+        </is>
+      </c>
+      <c r="G22" s="16" t="inlineStr">
+        <is>
+          <t>Luyện tập và thực hiện thành thạo thao tác chia nhánh tính năng dự án Web responsive, giải quyết nhuần nhuyễn xung đột mã nguồn bằng kỹ thuật debugging và ứng dụng thành công git stash trong tình huống phát triển thực tế.</t>
+        </is>
+      </c>
+      <c r="H22" s="16" t="inlineStr">
+        <is>
+          <t>CẤM: Quy trình Pull Request nhóm, Code Review, Git Flow nâng cao.</t>
+        </is>
+      </c>
+      <c r="I22" s="16" t="inlineStr">
+        <is>
+          <t>ĐÃ HỌC: Git CLI, GitHub Cloud, git branch, git merge, Merge Conflict, git stash, debugging cơ bản.</t>
+        </is>
+      </c>
+      <c r="J22" s="16" t="inlineStr">
+        <is>
+          <t>Git CLI 2.45+, GitHub Cloud (Conventional Commits, Git Flow, Semantic Branching)</t>
         </is>
       </c>
     </row>
     <row r="23" ht="24" customHeight="1">
-      <c r="A23" s="17" t="inlineStr">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>Session 07</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Lý thuyết</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>THEORY</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>Session 07 - Quy trình làm việc nâng cao, Debugging lịch sử &amp; Giao nhiệm vụ trên GitHub</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Lesson 01: Hoàn tác mã nguồn &amp; Kỹ thuật Debugging lịch sử Commit</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Phân biệt git reset (soft, mixed, hard) và git revert; Kỹ thuật debugging truy tìm commit gây lỗi bằng git log, git blame, git bisect; Chiến lược rollback an toàn trên kho chứa công khai.</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>Thực hiện hoàn tác mã nguồn an toàn với git revert/reset; Áp dụng thành công các công cụ debugging lịch sử commit để định vị nhanh đoạn code lỗi.</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>CẤM: Rebase nâng cao, GitHub Projects.</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>ĐÃ HỌC: Git CLI, commit history, merge conflict.</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>Git CLI 2.45+, GitHub Cloud (Conventional Commits, Git Flow, Semantic Branching)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="12" t="n"/>
+      <c r="B24" s="12" t="n"/>
+      <c r="C24" s="12" t="n"/>
+      <c r="D24" s="12" t="n"/>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Lesson 02: Quản lý kho chứa dự án JavaScript &amp; Tối ưu hóa Rebase</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Khái niệm Rebase; Phân biệt Git Rebase và Git Merge; Khi nào nên dùng rebase và khi nào không nên dùng; Cấu hình tối ưu lịch sử commit cho các project Web responsive sử dụng framework JavaScript; Lệnh git cherry-pick để trích xuất commit lẻ.</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>Phân biệt được sự khác nhau giữa git rebase và git merge; Áp dụng git cherry-pick để chọn lọc commit cần thiết vào nhánh sản phẩm của project framework.</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>CẤM: GitHub Issues.</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>ĐÃ HỌC: Phân nhánh, merge, hoàn tác commit.</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>Git CLI 2.45+, GitHub Cloud (Conventional Commits, Git Flow, Semantic Branching)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="13" t="n"/>
+      <c r="B25" s="13" t="n"/>
+      <c r="C25" s="13" t="n"/>
+      <c r="D25" s="13" t="n"/>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Lesson 03: Quản lý công việc &amp; Giao nhiệm vụ bằng GitHub Issues &amp; Projects</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Giới thiệu GitHub Issues và GitHub Projects; Kỹ thuật sinh issue, gắn label, milestone; Kỹ thuật giao nhiệm vụ (assignee) cho các thành viên trong nhóm; Liên kết commit và Pull Request với Issue bằng từ khóa (fixes #1, closes #2); Quy trình giao nộp và kiểm tra tiến độ mã nguồn.</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>Sinh và giao nhiệm vụ thành công cho các thành viên nhóm trên GitHub Projects; Liên kết chính xác commit/PR với Issue để quản lý tiến độ dự án.</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>CẤM: Thi cuối môn.</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>ĐÃ HỌC: GitHub Remote, Git Flow cơ bản.</t>
+        </is>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>Git CLI 2.45+, GitHub Cloud (Conventional Commits, Git Flow, Semantic Branching)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="24" customHeight="1">
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>Session 08</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>Mini project</t>
+        </is>
+      </c>
+      <c r="C26" s="17" t="inlineStr">
+        <is>
+          <t>MINI_PROJECT</t>
+        </is>
+      </c>
+      <c r="D26" s="18" t="inlineStr">
+        <is>
+          <t>Session 08 - Mini Project: Xây dựng kho lưu trữ mã nguồn Web nhóm chuẩn Git Flow</t>
+        </is>
+      </c>
+      <c r="E26" s="19" t="inlineStr">
+        <is>
+          <t>Session 08 - Mini Project: Xây dựng kho lưu trữ mã nguồn Web nhóm chuẩn Git Flow</t>
+        </is>
+      </c>
+      <c r="F26" s="19" t="inlineStr">
+        <is>
+          <t>Luyện tập làm việc nhóm (2-3 bạn/nhóm); Khởi tạo kho chứa nhóm trên GitHub Cloud cho dự án Web responsive xây dựng bằng framework JavaScript; Sinh và giao nhiệm vụ cụ thể cho từng thành viên qua GitHub Issues; Thiết lập mô hình phân nhánh Git Flow (main, develop, feature/*); Phân công công việc tích hợp các tính năng giao diện responsive; Thực hiện tạo Pull Request (PR) trên GitHub; Thực hiện Code Review, thảo luận, debugging xung đột logic và phê duyệt (Approve) PR để hợp nhất code vào nhánh develop; Sinh tài liệu phát hành và giao nộp mã nguồn hoàn thiện lên nhánh main.</t>
+        </is>
+      </c>
+      <c r="G26" s="19" t="inlineStr">
+        <is>
+          <t>Luyện tập xây dựng thành công kho lưu trữ mã nguồn chuẩn doanh nghiệp trên GitHub cho dự án Web responsive dùng framework JavaScript theo nhóm; Áp dụng nhuần nhuyễn mô hình Git Flow, sinh và phân công nhiệm vụ, tạo Pull Request và thực hiện Code Review thành công giữa các thành viên.</t>
+        </is>
+      </c>
+      <c r="H26" s="19" t="inlineStr">
+        <is>
+          <t>CẤM: Thi cuối môn.</t>
+        </is>
+      </c>
+      <c r="I26" s="19" t="inlineStr">
+        <is>
+          <t>ĐÃ HỌC: Toàn bộ kiến thức Git CLI, GitHub Cloud, Phân nhánh, Merge Conflict, Git Stash, Semantic Branching, Git Flow, Pull Request, Debugging, GitHub Issues &amp; Projects.</t>
+        </is>
+      </c>
+      <c r="J26" s="19" t="inlineStr">
+        <is>
+          <t>Git CLI 2.45+, GitHub Cloud (Conventional Commits, Git Flow, Semantic Branching)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="10" t="inlineStr">
         <is>
           <t>Session 09</t>
         </is>
       </c>
-      <c r="B23" s="17" t="inlineStr">
-        <is>
-          <t>Mini project</t>
-        </is>
-      </c>
-      <c r="C23" s="17" t="inlineStr">
-        <is>
-          <t>MINI_PROJECT</t>
-        </is>
-      </c>
-      <c r="D23" s="18" t="inlineStr">
-        <is>
-          <t>Session 09 - Dự án nhóm phối hợp Git Flow</t>
-        </is>
-      </c>
-      <c r="E23" s="19" t="inlineStr">
-        <is>
-          <t>Session 09 - Dự án nhóm phối hợp Git Flow</t>
-        </is>
-      </c>
-      <c r="F23" s="19" t="inlineStr">
-        <is>
-          <t>Git Flow; Pull Request; Conflict; GitHub CLI</t>
-        </is>
-      </c>
-      <c r="G23" s="19" t="inlineStr">
-        <is>
-          <t>Hoàn thành dự án nhóm có giải quyết conflict.</t>
-        </is>
-      </c>
-      <c r="H23" s="19" t="inlineStr">
-        <is>
-          <t>CẤM: Push thẳng lên nhánh main.</t>
-        </is>
-      </c>
-      <c r="I23" s="19" t="inlineStr">
-        <is>
-          <t>ĐÃ HỌC: Git Flow, PR, giải quyết conflict.</t>
-        </is>
-      </c>
-      <c r="J23" s="19" t="inlineStr">
-        <is>
-          <t>Git 2.45+, GitHub Web &amp; CLI, Git Flow Standard Branching Model, SSH / GPG Standard Authentication (Conventional Commits, Clean Git History, .gitignore Best Practices)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="24" customHeight="1">
-      <c r="A24" s="20" t="inlineStr">
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>Lý thuyết</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>THEORY</t>
+        </is>
+      </c>
+      <c r="D27" s="11" t="inlineStr">
+        <is>
+          <t>Session 09 - Cài đặt, Cấu hình môi trường nâng cao &amp; Ôn tập chuẩn hóa mã nguồn</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Lesson 01: Giới thiệu quy trình Git Flow &amp; Kỹ thuật debugging logic mã nguồn</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Giới thiệu tổng quan quy trình Git Flow làm việc nhóm; Lý thuyết debugging mã nguồn khi xảy ra sai lệch phiên bản trong dự án Web framework; Nguyên lý truy vết commit lỗi bằng git reflog.</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>Trình bày được quy trình Git Flow chuẩn và nguyên lý debugging mã nguồn bằng git reflog.</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>CẤM: Thao tác trực tiếp bài thi cuối môn.</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>ĐÃ HỌC: Các lệnh Git CLI, Branching, Rebase, Stash, GitHub Issues.</t>
+        </is>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>Git CLI 2.45+, GitHub Cloud (Conventional Commits, Git Flow, Semantic Branching)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="12" t="n"/>
+      <c r="B28" s="12" t="n"/>
+      <c r="C28" s="12" t="n"/>
+      <c r="D28" s="12" t="n"/>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Lesson 02: Cài đặt &amp; Cấu hình môi trường kho lưu trữ chuẩn doanh nghiệp</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Cài đặt và cấu hình môi trường repository chuyên nghiệp: cấu hình file .gitignore tối ưu cho dự án framework, sinh file README.md theo chuẩn Markdown, thiết lập tài liệu CONTRIBUTING.md và cấu hình môi trường làm việc Git.</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>Thực hiện cài đặt, sinh tự động và cấu hình thành công các tệp tin môi trường kho lưu trữ đạt chuẩn doanh nghiệp.</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>CẤM: Thao tác bài thi cuối môn.</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>ĐÃ HỌC: Giới thiệu Git Flow, Git CLI cơ bản.</t>
+        </is>
+      </c>
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>Git CLI 2.45+, GitHub Cloud (Conventional Commits, Git Flow, Semantic Branching)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="24" customHeight="1">
+      <c r="A29" s="13" t="n"/>
+      <c r="B29" s="13" t="n"/>
+      <c r="C29" s="13" t="n"/>
+      <c r="D29" s="13" t="n"/>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Lesson 03: Kiểm tra &amp; Thực thao tác dọn dẹp kho chứa mã nguồn</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Kiểm tra tính toàn vẹn của kho chứa mã nguồn; Thực thao tác dọn dẹp nhánh rác, kiểm tra lịch sử commit và hướng dẫn quy chuẩn giao nộp bài thi cuối môn.</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>Thực hiện kiểm tra và dọn dẹp thành công kho lưu trữ mã nguồn; Thao tác chính xác quy trình giao nộp bài thi cuối môn.</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>CẤM: Làm bài thi cuối môn trước thời hạn.</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>ĐÃ HỌC: Cài đặt và cấu hình môi trường kho lưu trữ.</t>
+        </is>
+      </c>
+      <c r="J29" s="5" t="inlineStr">
+        <is>
+          <t>Git CLI 2.45+, GitHub Cloud (Conventional Commits, Git Flow, Semantic Branching)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" s="20" t="inlineStr">
         <is>
           <t>Session 10</t>
         </is>
       </c>
-      <c r="B24" s="20" t="inlineStr">
+      <c r="B30" s="20" t="inlineStr">
         <is>
           <t>Thi cuối môn</t>
         </is>
       </c>
-      <c r="C24" s="20" t="inlineStr">
+      <c r="C30" s="20" t="inlineStr">
         <is>
           <t>FINAL</t>
         </is>
       </c>
-      <c r="D24" s="21" t="inlineStr">
-        <is>
-          <t>Session 10 - Thi thực hành quản lý mã nguồn</t>
-        </is>
-      </c>
-      <c r="E24" s="22" t="inlineStr">
-        <is>
-          <t>Session 10 - Thi thực hành quản lý mã nguồn</t>
-        </is>
-      </c>
-      <c r="F24" s="22" t="inlineStr">
-        <is>
-          <t>Git CLI; GitHub; Git Flow; Pull Request</t>
-        </is>
-      </c>
-      <c r="G24" s="22" t="inlineStr">
-        <is>
-          <t>Hoàn thành bài thi quản lý mã nguồn chuẩn.</t>
-        </is>
-      </c>
-      <c r="H24" s="22" t="inlineStr">
-        <is>
-          <t>CẤM: Sử dụng tài liệu không được phép.</t>
-        </is>
-      </c>
-      <c r="I24" s="22" t="inlineStr">
-        <is>
-          <t>ĐÃ HỌC: Toàn bộ nội dung Git trong khóa học.</t>
-        </is>
-      </c>
-      <c r="J24" s="22" t="inlineStr">
-        <is>
-          <t>Git 2.45+, GitHub Web &amp; CLI, Git Flow Standard Branching Model, SSH / GPG Standard Authentication (Conventional Commits, Clean Git History, .gitignore Best Practices)</t>
+      <c r="D30" s="21" t="inlineStr">
+        <is>
+          <t>Session 10 - Thi cuối môn: Quản lý phiên bản &amp; Phối hợp mã nguồn Git</t>
+        </is>
+      </c>
+      <c r="E30" s="22" t="inlineStr">
+        <is>
+          <t>Session 10 - Thi cuối môn: Quản lý phiên bản &amp; Phối hợp mã nguồn Git</t>
+        </is>
+      </c>
+      <c r="F30" s="22" t="inlineStr">
+        <is>
+          <t>Bài thi thực hành cá nhân/nhóm trên máy tính: Khởi tạo Git repository cho một dự án Web responsive phát triển trên framework JavaScript cho trước; Cấu hình .gitignore và commit theo chuẩn Conventional Commits; Đẩy repository lên GitHub Cloud; Thực hiện phân nhánh tính năng (feature branch); Giả lập, debugging và giải quyết các tình huống xung đột mã nguồn (Merge Conflict); Tạo Pull Request, sinh issue giao nhiệm vụ, thực hiện Code Review và giao nộp mã nguồn hoàn chỉnh vào nhánh main/develop.</t>
+        </is>
+      </c>
+      <c r="G30" s="22" t="inlineStr">
+        <is>
+          <t>Hoàn thành 100% yêu cầu bài thi thực hành; Chứng tỏ năng lực thao tác thành thạo Git CLI và GitHub Cloud trong việc lưu trữ, quản lý phiên bản dự án Web responsive, debugging mã nguồn và phối hợp dự án đạt chuẩn doanh nghiệp.</t>
+        </is>
+      </c>
+      <c r="H30" s="22" t="inlineStr">
+        <is>
+          <t>CẤM: Can thiệp mã nguồn sau giờ làm bài.</t>
+        </is>
+      </c>
+      <c r="I30" s="22" t="inlineStr">
+        <is>
+          <t>ĐÃ HỌC: Toàn bộ kiến thức và kỹ năng môn IT-105.</t>
+        </is>
+      </c>
+      <c r="J30" s="22" t="inlineStr">
+        <is>
+          <t>Git CLI 2.45+, GitHub Cloud (Conventional Commits, Git Flow, Semantic Branching)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="23">
-    <mergeCell ref="A12:A14"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="C12:C14"/>
-    <mergeCell ref="D12:D14"/>
-    <mergeCell ref="A20:A22"/>
+  <mergeCells count="27">
+    <mergeCell ref="C27:C29"/>
+    <mergeCell ref="C9:C13"/>
+    <mergeCell ref="D15:D17"/>
+    <mergeCell ref="B9:B13"/>
+    <mergeCell ref="B18:B21"/>
     <mergeCell ref="B1:J1"/>
-    <mergeCell ref="D8:D10"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="B20:B22"/>
-    <mergeCell ref="D20:D22"/>
-    <mergeCell ref="B16:B18"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="B12:B14"/>
-    <mergeCell ref="C20:C22"/>
-    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="B15:B17"/>
+    <mergeCell ref="A23:A25"/>
+    <mergeCell ref="C23:C25"/>
+    <mergeCell ref="D23:D25"/>
+    <mergeCell ref="D9:D13"/>
+    <mergeCell ref="A9:A13"/>
+    <mergeCell ref="A15:A17"/>
+    <mergeCell ref="C6:C8"/>
+    <mergeCell ref="D6:D8"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="D18:D21"/>
+    <mergeCell ref="C15:C17"/>
+    <mergeCell ref="D27:D29"/>
+    <mergeCell ref="A6:A8"/>
+    <mergeCell ref="B27:B29"/>
+    <mergeCell ref="B23:B25"/>
     <mergeCell ref="B3:J3"/>
-    <mergeCell ref="A16:A18"/>
-    <mergeCell ref="C16:C18"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="D16:D18"/>
-    <mergeCell ref="C8:C10"/>
-    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="A27:A29"/>
+    <mergeCell ref="B6:B8"/>
     <mergeCell ref="B2:J2"/>
+    <mergeCell ref="C18:C21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>